<commit_message>
feat: 86-company real prospect list (4 research agents) + invoice generator + €15k MRR plan
prospects-master.csv: 86 evidenced EU/SG/UAE high-risk AI companies (33 Tier-A) across
HR-tech/fintech/insurtech/legal-tech/health-tech, each w/ use-case hook + why-now signal.
Loaded into tracker; outreach wave generated (86 personalized msg sets).
build_invoice.py: Payoneer-ready invoice PDF (founding/starter/annual/report) — turns yes->cash.
PATH-TO-15K-MRR.md: pricing ladder (Starter EUR490 / Founding $1,500 / Enterprise) + funnel math.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gtm/07-sprint/Verispect-Sprint-Tracker.xlsx
+++ b/gtm/07-sprint/Verispect-Sprint-Tracker.xlsx
@@ -1331,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1425,14 +1425,14 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Empion</t>
+          <t>Maki People</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr"/>
       <c r="D3" s="5" t="inlineStr"/>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Berlin DE</t>
+          <t>Paris FR</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>AI culture/skills matching for recruitment</t>
+          <t>Conversational AI assesses skills &amp; filters candidates</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr"/>
@@ -1457,7 +1457,11 @@
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr"/>
-      <c r="L3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>€27.8M Series A; H&amp;M/BNP/PwC clients</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1467,14 +1471,14 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Beamery</t>
+          <t>HrFlow.ai</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr"/>
       <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Paris FR</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -1484,12 +1488,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>AI talent matching &amp; candidate ranking</t>
+          <t>Explainable AI scores &amp; prioritizes candidate profiles</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr"/>
@@ -1499,7 +1503,11 @@
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>€6M pre-A Apr 2026; explainability angle</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1509,14 +1517,14 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Textkernel</t>
+          <t>Dex</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="5" t="inlineStr"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Amsterdam NL</t>
+          <t>London UK</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -1526,12 +1534,12 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>CV parsing &amp; job matching (ML/LLM)</t>
+          <t>AI matches engineers to roles via ML engine</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr"/>
@@ -1541,7 +1549,11 @@
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr"/>
-      <c r="L5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>$5.3M seed Apr 2026 (a16z Speedrun)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1551,14 +1563,14 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Equalture</t>
+          <t>Carv</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Rotterdam NL</t>
+          <t>Amsterdam NL</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -1568,12 +1580,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Bias-aware hiring assessments</t>
+          <t>AI pre-screens candidates via chat/voice</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr"/>
@@ -1583,7 +1595,11 @@
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>$10M seed; launched 2024</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1593,14 +1609,14 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Tengai</t>
+          <t>Empion</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr"/>
       <c r="D7" s="5" t="inlineStr"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Stockholm SE</t>
+          <t>Berlin DE</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -1610,12 +1626,12 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Unbiased AI interview screening</t>
+          <t>AI robo-advisor matches/ranks candidates</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr"/>
@@ -1625,7 +1641,11 @@
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>~€9M raised; acquired Zalvus</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1652,12 +1672,12 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>AI video interview / behavioral scoring</t>
+          <t>Video AI infers personality to assess fit</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
@@ -1667,24 +1687,28 @@
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>€9M Series A; behavioral scoring = high scrutiny</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>HeroHunt.ai</t>
+          <t>Tengai</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Stockholm SE</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1694,12 +1718,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>LLM candidate sourcing</t>
+          <t>AI interview avatar screens candidates unbiased</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
@@ -1709,24 +1733,28 @@
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Brand = unbiased; needs evidence</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>SmartRecruiters</t>
+          <t>Vinter</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>EU/US</t>
+          <t>London UK</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1736,12 +1764,12 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>AI candidate screening in ATS</t>
+          <t>AI evaluates candidates across tasks &amp; video</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
@@ -1751,7 +1779,11 @@
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr"/>
-      <c r="L10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>€1.4M seed; 'bias-free' positioning</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1761,14 +1793,14 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Honeypot</t>
+          <t>Alva Labs</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr"/>
       <c r="D11" s="5" t="inlineStr"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Berlin DE</t>
+          <t>Stockholm SE</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1778,12 +1810,12 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Dev hiring marketplace + matching</t>
+          <t>AI psychometric tests predict candidate fit</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
@@ -1793,7 +1825,11 @@
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr"/>
-      <c r="L11" s="5" t="inlineStr"/>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>$14.2M Series A (VNV Global)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1803,14 +1839,14 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Personio</t>
+          <t>Sapia.ai</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Munich DE</t>
+          <t>London UK (ops)</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1820,12 +1856,12 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>HR platform adding AI features</t>
+          <t>Chat AI interviews score &amp; shortlist candidates</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr"/>
@@ -1835,39 +1871,43 @@
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr"/>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>10M+ interviews; HQ AU - flag</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Taktile</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr"/>
       <c r="D13" s="5" t="inlineStr"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Berlin DE</t>
+          <t>London UK</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Automated credit/risk decisioning</t>
+          <t>Debiased task-based candidate assessments</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
@@ -1877,39 +1917,43 @@
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr"/>
-      <c r="L13" s="5" t="inlineStr"/>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>BIT spin-out; public RAI claim</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Abound</t>
+          <t>Maki/Neobrain</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr"/>
       <c r="D14" s="5" t="inlineStr"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Paris FR</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>AI consumer credit underwriting</t>
+          <t>AI maps skills &amp; assesses employees for mobility</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
@@ -1919,39 +1963,43 @@
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr"/>
-      <c r="L14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>€20M Series A (Breega)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Lendable</t>
+          <t>AssessFirst</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr"/>
       <c r="D15" s="5" t="inlineStr"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Paris FR</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>ML credit/lending decisions</t>
+          <t>AI predicts candidate potential</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr"/>
@@ -1961,39 +2009,43 @@
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr"/>
-      <c r="L15" s="5" t="inlineStr"/>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>3500+ companies 40+ countries</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Kennek</t>
+          <t>Orbio</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="5" t="inlineStr"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Madrid ES</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Lending operations / underwriting</t>
+          <t>Autonomous AI agents run screening end-to-end</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr"/>
@@ -2003,7 +2055,11 @@
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr"/>
-      <c r="L16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>€6.4M raised; founded 2025</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2013,29 +2069,29 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Solaris</t>
+          <t>Wrksense</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr"/>
       <c r="D17" s="5" t="inlineStr"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Berlin DE</t>
+          <t>Dublin IE</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Banking-as-a-service + risk models</t>
+          <t>Full AI recruiter screens/evaluates candidates</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr"/>
@@ -2045,7 +2101,11 @@
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr"/>
-      <c r="L17" s="5" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Targets orgs hiring 200+/yr</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2055,29 +2115,29 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Scalable Capital</t>
+          <t>HrFlow/Carv tier</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr"/>
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Munich DE</t>
+          <t>Rotterdam NL</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Robo-advisory / risk profiling</t>
+          <t>AI matching students/pros to employers (Magnet.me)</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr"/>
@@ -2087,39 +2147,43 @@
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr"/>
-      <c r="L18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>400k+ professionals</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Akur8</t>
+          <t>TestGorilla</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr"/>
       <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Paris FR</t>
+          <t>Amsterdam NL</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Insurtech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>ML insurance pricing/underwriting</t>
+          <t>AI skills assessments + resume scoring</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr"/>
@@ -2129,39 +2193,43 @@
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr"/>
-      <c r="L19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Large skills-test library</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Shift Technology</t>
+          <t>Globus.ai</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr"/>
       <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Paris FR</t>
+          <t>Oslo NO</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Insurtech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>AI claims &amp; fraud decisioning</t>
+          <t>AI matches &amp; books healthcare staff</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr"/>
@@ -2171,39 +2239,43 @@
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr"/>
-      <c r="L20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>$4.8M seed; 12x growth</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>wefox</t>
+          <t>Beamery</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr"/>
       <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Berlin DE</t>
+          <t>London UK</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Insurtech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>AI claims/underwriting assist</t>
+          <t>AI infers skills to match/rank talent</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr"/>
@@ -2213,39 +2285,43 @@
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr"/>
-      <c r="L21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Enterprise clients; runs large</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Getsafe</t>
+          <t>HeyJobs</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr"/>
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Heidelberg DE</t>
+          <t>Berlin DE</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Insurtech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>AI claims automation</t>
+          <t>ML matching scores candidate shortlists</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr"/>
@@ -2255,39 +2331,43 @@
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr"/>
-      <c r="L22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>$59M raised; runs large</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Zego</t>
+          <t>Job&amp;Talent</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr"/>
       <c r="D23" s="5" t="inlineStr"/>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Madrid ES</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Insurtech</t>
+          <t>HR-tech</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Usage-based pricing ML</t>
+          <t>ML automates blue-collar hiring/matching</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr"/>
@@ -2297,7 +2377,11 @@
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr"/>
-      <c r="L23" s="5" t="inlineStr"/>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>One of EU's largest; runs large</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2307,29 +2391,29 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Robin AI</t>
+          <t>Taktile</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr"/>
       <c r="D24" s="5" t="inlineStr"/>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Berlin DE</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Legal-tech</t>
+          <t>Fintech</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>LLM contract review &amp; risk</t>
+          <t>AI credit/risk underwriting decision platform</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr"/>
@@ -2339,7 +2423,11 @@
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr"/>
-      <c r="L24" s="5" t="inlineStr"/>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>$54M Series B Feb 2025; 24 markets</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2349,29 +2437,29 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Leya</t>
+          <t>Banxware</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr"/>
       <c r="D25" s="5" t="inlineStr"/>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Stockholm SE</t>
+          <t>Berlin DE</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Legal-tech</t>
+          <t>Fintech</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>LLM legal research/review</t>
+          <t>AI underwriting for embedded SME lending</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr"/>
@@ -2381,7 +2469,11 @@
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr"/>
-      <c r="L25" s="5" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>€10M from UniCredit Jun 2025</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2391,29 +2483,29 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Luminance</t>
+          <t>Karmen</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr"/>
       <c r="D26" s="5" t="inlineStr"/>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Cambridge UK</t>
+          <t>Paris FR</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Legal-tech</t>
+          <t>Fintech</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>AI contract analysis</t>
+          <t>AI credit-risk scoring for revenue-based finance</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr"/>
@@ -2423,39 +2515,43 @@
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr"/>
-      <c r="L26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>$9.4M Jan 2025 (Bpifrance)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Genie AI</t>
+          <t>Defacto</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr"/>
       <c r="D27" s="5" t="inlineStr"/>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Paris FR</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Legal-tech</t>
+          <t>Fintech</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>LLM legal drafting/review</t>
+          <t>Automated AI credit decisioning for SME lending</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr"/>
@@ -2465,39 +2561,43 @@
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr"/>
-      <c r="L27" s="5" t="inlineStr"/>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>€16M; €167M Citi facility</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Juro</t>
+          <t>Mifundo</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr"/>
       <c r="D28" s="5" t="inlineStr"/>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Tallinn EE</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Legal-tech</t>
+          <t>Fintech</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Contract automation + AI</t>
+          <t>AI cross-border credit scoring</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr"/>
@@ -2507,17 +2607,21 @@
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr"/>
-      <c r="L28" s="5" t="inlineStr"/>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>€10M EIC Sep 2024; EU credit-passport</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Definely</t>
+          <t>Plend</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr"/>
@@ -2529,17 +2633,17 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Legal-tech</t>
+          <t>Fintech</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Contract drafting AI</t>
+          <t>Open-banking + AI affordability/credit scoring</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr"/>
@@ -2549,7 +2653,11 @@
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr"/>
-      <c r="L29" s="5" t="inlineStr"/>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>£40M seed; ClearScore partnership</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2559,29 +2667,29 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Bayzat</t>
+          <t>Baobab Insurance</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr"/>
       <c r="D30" s="5" t="inlineStr"/>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Dubai UAE</t>
+          <t>Berlin DE</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>HR-tech</t>
+          <t>Insurtech</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>HR &amp; payroll + AI features</t>
+          <t>AI-native cyber-risk underwriting</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr"/>
@@ -2591,7 +2699,11 @@
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr"/>
-      <c r="L30" s="5" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>€12M Series A Jun 2025</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -2601,29 +2713,29 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>ADVANCE.AI</t>
+          <t>Qantev</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr"/>
       <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Paris FR</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>Insurtech</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>AI KYC + credit scoring (APAC)</t>
+          <t>AI claims platform for health/life insurers</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr"/>
@@ -2633,39 +2745,43 @@
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr"/>
-      <c r="L31" s="5" t="inlineStr"/>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>€30M Oct 2024 (Blossom)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Kredivo / FinAccel</t>
+          <t>Sprout.ai</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr"/>
       <c r="D32" s="5" t="inlineStr"/>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>London UK</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>Insurtech</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>AI consumer credit (SEA)</t>
+          <t>GenAI/LLM claims assessment automation</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr"/>
@@ -2675,39 +2791,43 @@
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr"/>
-      <c r="L32" s="5" t="inlineStr"/>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>£5.4M; patented LLM claims tech</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Lenddo</t>
+          <t>ClaimSorted</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr"/>
       <c r="D33" s="5" t="inlineStr"/>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>London UK</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Fintech</t>
+          <t>Insurtech</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Alt-data credit scoring</t>
+          <t>AI claims-handling automation (TPA)</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
@@ -2717,7 +2837,11 @@
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr"/>
-      <c r="L33" s="5" t="inlineStr"/>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>€11.4M seed Oct 2025</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2727,29 +2851,29 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>G42</t>
+          <t>SME Finance</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr"/>
       <c r="D34" s="5" t="inlineStr"/>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Abu Dhabi UAE</t>
+          <t>Vilnius LT</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>AI/Enterprise</t>
+          <t>Fintech</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Enterprise AI incl regulated use</t>
+          <t>AI lending decisions for SMEs &lt;1hr</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr"/>
@@ -2759,7 +2883,11 @@
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr"/>
-      <c r="L34" s="5" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>€40M InvestEU/EIF facility</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -2769,14 +2897,14 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Sava</t>
+          <t>Creamfinance</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr"/>
       <c r="D35" s="5" t="inlineStr"/>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Dubai UAE</t>
+          <t>Warsaw PL</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -2786,12 +2914,12 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>SME spend/credit AI</t>
+          <t>ML consumer credit scoring on alt-data</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
@@ -2801,24 +2929,28 @@
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr"/>
-      <c r="L35" s="5" t="inlineStr"/>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>5-market scoring engine</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Tractable</t>
+          <t>Bdeo</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr"/>
       <c r="D36" s="5" t="inlineStr"/>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>London UK</t>
+          <t>Madrid ES</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -2828,12 +2960,12 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>AI visual claims assessment</t>
+          <t>AI visual intelligence for motor claims</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr"/>
@@ -2843,39 +2975,43 @@
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr"/>
-      <c r="L36" s="5" t="inlineStr"/>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>&gt;50% Spanish motor underwriting</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>HireVue</t>
+          <t>Cleverea</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr"/>
       <c r="D37" s="5" t="inlineStr"/>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>US/EU</t>
+          <t>Barcelona ES</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>HR-tech</t>
+          <t>Insurtech</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>AI video interview assessment</t>
+          <t>ML underwriting &amp; fraud (neo-insurer)</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr"/>
@@ -2885,39 +3021,43 @@
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr"/>
-      <c r="L37" s="5" t="inlineStr"/>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>€5M seed (Stride)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Personio/others</t>
+          <t>omni:us</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr"/>
       <c r="D38" s="5" t="inlineStr"/>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>Berlin DE</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>HR-tech</t>
+          <t>Insurtech</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI end-to-end claims automation</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>seed/WebSearch</t>
+          <t>agent-research</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr"/>
@@ -2927,33 +3067,2309 @@
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr"/>
-      <c r="L38" s="5" t="inlineStr"/>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Wurttembergische partnership</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n"/>
-      <c r="B39" s="5" t="n"/>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="5" t="n"/>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="n"/>
-      <c r="K39" s="5" t="n"/>
-      <c r="L39" s="5" t="n"/>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>MarvelX</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr"/>
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Amsterdam NL</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>AI claims/workflow automation + fraud</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr"/>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr"/>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>€5.4M (EQT Ventures) May 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Monto (Capcito)</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr"/>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Stockholm SE</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Real-time AI scoring for SME credit</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr"/>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr"/>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Powers SME lender decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>INSRD</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Berlin DE</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Industry AI for SME risk/underwriting</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr"/>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>€500k pre-seed; early fit</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Status values: New · Touched · Replied · Snapshot · Demo · WON · Lost · Nurture</t>
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Elucidate</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Berlin DE</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>ML financial-crime risk scoring for FIs</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr"/>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr"/>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>~€8M Series A; regulated FIs</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Tier A = high-risk vertical + recent raise + EU (hit first). B = good fit. C = backup/Tier-2.</t>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Surebird</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Amsterdam NL</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>AI insurance underwriting/ops automation</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr"/>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr"/>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>Recent funding; early-stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Akur8</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Paris FR</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>ML actuarial pricing &amp; reserving</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr"/>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr"/>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>$120M Series C; 300+ insurers</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Descartes Underwriting</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Paris FR</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>AI parametric risk underwriting</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr"/>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr"/>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>$120M Series B; Generali</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Abound</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>London UK</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>AI cashflow underwriting on Open Banking</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr"/>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr"/>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>£250M Deutsche Bank facility</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Robin AI</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr"/>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>London UK</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>LLM contract review (2M+ contracts)</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr"/>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr"/>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>$26M Series B+ Nov 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Genie AI</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>London UK</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>LLM drafting + review of legal docs</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr"/>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr"/>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>$17.8M Series A (GV) Oct 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Leya</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr"/>
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Stockholm SE</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>LLM assistant review/search/drafting</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr"/>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>$25M Series A (Redpoint); 70+ firms</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Garfield AI</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr"/>
+      <c r="D50" s="5" t="inlineStr"/>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>London UK</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>LLM litigation assistant (debt recovery)</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr"/>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr"/>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>First SRA-authorised AI law firm 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Noxtua</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Berlin DE</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Sovereign legal LLM (German law)</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr"/>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr"/>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>€80.7M Series B (C.H. Beck)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Definely</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr"/>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>London UK</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>AI contract drafting/review (Cascade)</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr"/>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr"/>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>Magic Circle clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Luminance</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Cambridge UK</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>Proprietary LLM contract review</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr"/>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr"/>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>$75M Series C; runs large</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>LawX</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr"/>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Berlin DE</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>AI OS / back-office layer for legal</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr"/>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr"/>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>€7.5M (Motive Partners)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Tomorro</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr"/>
+      <c r="D55" s="5" t="inlineStr"/>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Paris FR</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>AI contract drafting/negotiation (CLM)</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr"/>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr"/>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>France Legaltech program</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Saga</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr"/>
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Amsterdam NL</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>Agentic LLM legal work assistants</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr"/>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K56" s="5" t="inlineStr"/>
+      <c r="L56" s="5" t="inlineStr">
+        <is>
+          <t>€1.5M+ seed Oct 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Henchman</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Ghent BE</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>GPT contract drafting/clause retrieval</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr"/>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr"/>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>Acquired by LexisNexis Jun 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Brightflag</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr"/>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Dublin IE</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Legal-tech</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>AI legal-spend analysis &amp; matter classification</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr"/>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K58" s="5" t="inlineStr"/>
+      <c r="L58" s="5" t="inlineStr">
+        <is>
+          <t>NLP on legal data; Series A+</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>TORTUS AI</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr"/>
+      <c r="D59" s="5" t="inlineStr"/>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>London UK</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Health-tech</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>GenAI ambient clinical scribe</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr"/>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K59" s="5" t="inlineStr"/>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>Largest NHS AI-scribe trial 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Anima Health</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr"/>
+      <c r="D60" s="5" t="inlineStr"/>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>London UK</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Health-tech</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>AI clinical triage &amp; care-navigation</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr"/>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K60" s="5" t="inlineStr"/>
+      <c r="L60" s="5" t="inlineStr">
+        <is>
+          <t>$12M Series A (Molten); 300+ NHS practices</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Corti</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr"/>
+      <c r="D61" s="5" t="inlineStr"/>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Copenhagen DK</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Health-tech</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>Clinical-reasoning LLM for consultations</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr"/>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr"/>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>Launched FactsR agentic reasoning Jun 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Visiba Care</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Gothenburg SE</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Health-tech</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>AI symptom triage (CE-marked device)</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr"/>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr">
+        <is>
+          <t>Deployed in NHS 111</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Klinik</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr"/>
+      <c r="D63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Helsinki FI</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Health-tech</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>AI total-triage 1000+ symptoms</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr"/>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K63" s="5" t="inlineStr"/>
+      <c r="L63" s="5" t="inlineStr">
+        <is>
+          <t>CE-marked; EU+UK expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Symptoma</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr"/>
+      <c r="D64" s="5" t="inlineStr"/>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Salzburg AT</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Health-tech</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>AI symptom checker 20k+ diseases</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr"/>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K64" s="5" t="inlineStr"/>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>In NHS AI-triage landscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Mediktor</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr"/>
+      <c r="D65" s="5" t="inlineStr"/>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Barcelona ES</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Health-tech</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>LLM conversational digital triage</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr"/>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="inlineStr"/>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>Clinically validated LLM triage</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Quibim</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr"/>
+      <c r="D66" s="5" t="inlineStr"/>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Valencia ES</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Health-tech</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>AI radiology/imaging biomarkers</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr"/>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="inlineStr"/>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>$50M Series A; 170+ installations</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>X0PA AI</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr"/>
+      <c r="D67" s="5" t="inlineStr"/>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>HR-tech</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>AI screens/ranks/scores candidates</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr"/>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K67" s="5" t="inlineStr"/>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>Endorsed by SG AI Verify; Samsung/gov clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>finbots.ai</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>creditX AI builds credit-risk scorecards</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr"/>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K68" s="5" t="inlineStr"/>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>MAS Veritas + AI Verify; digital-bank client</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Tabby</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr"/>
+      <c r="D69" s="5" t="inlineStr"/>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Dubai UAE</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>Real-time AI underwriting at checkout (BNPL)</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr"/>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="inlineStr"/>
+      <c r="L69" s="5" t="inlineStr">
+        <is>
+          <t>$160M Series E at $3.3B; IPO underway</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Bayzat</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr"/>
+      <c r="D70" s="5" t="inlineStr"/>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Dubai UAE</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>HR-tech</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>HR/payroll AI + anomaly detection</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr"/>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="inlineStr"/>
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>$60M+ (Point72/Mubadala); 4000+ companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Igloo</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr"/>
+      <c r="D71" s="5" t="inlineStr"/>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>Real-time risk + AI underwriting/claims</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr"/>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K71" s="5" t="inlineStr"/>
+      <c r="L71" s="5" t="inlineStr">
+        <is>
+          <t>~$100M raised; AI-native by 2026; Tokio Marine</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>NymCard</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr"/>
+      <c r="D72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi UAE</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>AI credit decisioning + loan servicing</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr"/>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr"/>
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>Central Bank UAE licensed; MENA embedded lending</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Tamara</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr"/>
+      <c r="D73" s="5" t="inlineStr"/>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Riyadh SA</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>Shariah BNPL credit/risk decisioning</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr"/>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="inlineStr"/>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>$2.4B facility (Goldman/Citi/Apollo); 20M customers</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>HireQuotient</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr"/>
+      <c r="D74" s="5" t="inlineStr"/>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>HR-tech</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>AI recruiting OS: sourcing/assessment/video scoring</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr"/>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr"/>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>Growth-stage; agentic recruiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Fuku AI</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr"/>
+      <c r="D75" s="5" t="inlineStr"/>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>HR-tech</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>AI sources/screens/evaluates interviews</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr"/>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K75" s="5" t="inlineStr"/>
+      <c r="L75" s="5" t="inlineStr">
+        <is>
+          <t>Recently launched in SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>CredoLab</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr"/>
+      <c r="D76" s="5" t="inlineStr"/>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>Credit scorecards from smartphone metadata</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr"/>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="inlineStr"/>
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t>50+ lenders 15 countries; Visa/CIMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Trusting Social</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr"/>
+      <c r="D77" s="5" t="inlineStr"/>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>AI credit scores from alt-data</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr"/>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K77" s="5" t="inlineStr"/>
+      <c r="L77" s="5" t="inlineStr">
+        <is>
+          <t>Sequoia/Tencent-backed</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>LenddoEFL</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr"/>
+      <c r="D78" s="5" t="inlineStr"/>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>AI/behavioral-data credit scoring</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr"/>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="inlineStr"/>
+      <c r="L78" s="5" t="inlineStr">
+        <is>
+          <t>5M+ assessments; $2B+ disbursed</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Funding Societies</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr"/>
+      <c r="D79" s="5" t="inlineStr"/>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>AI credit models underwrite SME loans</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr"/>
+      <c r="J79" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K79" s="5" t="inlineStr"/>
+      <c r="L79" s="5" t="inlineStr">
+        <is>
+          <t>SE Asia's largest SME lender; $4B+</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Aspire</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr"/>
+      <c r="D80" s="5" t="inlineStr"/>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>Aspire AI + ML credit decisioning</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr"/>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="inlineStr"/>
+      <c r="L80" s="5" t="inlineStr">
+        <is>
+          <t>Launched Aspire AI; Singlife partner</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Beehive</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr"/>
+      <c r="D81" s="5" t="inlineStr"/>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Dubai UAE</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>AI + alt-data SME borrower scoring</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr"/>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K81" s="5" t="inlineStr"/>
+      <c r="L81" s="5" t="inlineStr">
+        <is>
+          <t>e&amp; majority stake; DFSA-regulated</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Lendo</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr"/>
+      <c r="D82" s="5" t="inlineStr"/>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>Riyadh SA</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>AI screens SME borrowers (debt crowdfunding)</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr"/>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K82" s="5" t="inlineStr"/>
+      <c r="L82" s="5" t="inlineStr">
+        <is>
+          <t>~$740M financing 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Tookitaki</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr"/>
+      <c r="D83" s="5" t="inlineStr"/>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>AI risk engine for AML/KYC due diligence</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr"/>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K83" s="5" t="inlineStr"/>
+      <c r="L83" s="5" t="inlineStr">
+        <is>
+          <t>MAS-aligned; enterprise banks</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Cynopsis</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr"/>
+      <c r="D84" s="5" t="inlineStr"/>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>AI KYC/AML + identity screening</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr"/>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K84" s="5" t="inlineStr"/>
+      <c r="L84" s="5" t="inlineStr">
+        <is>
+          <t>Regulated-FI base across APAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Bolttech</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr"/>
+      <c r="D85" s="5" t="inlineStr"/>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>AI/ML embedded insurance risk/claims</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr"/>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K85" s="5" t="inlineStr"/>
+      <c r="L85" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech unicorn; global insurers</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Hala (Addenda)</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr"/>
+      <c r="D86" s="5" t="inlineStr"/>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi UAE</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>AI/ML motor underwriting &amp; pricing</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr"/>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K86" s="5" t="inlineStr"/>
+      <c r="L86" s="5" t="inlineStr">
+        <is>
+          <t>$5M (Mubadala); ADGM-licensed</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Yallacompare</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr"/>
+      <c r="D87" s="5" t="inlineStr"/>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>Dubai UAE</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>Engine matches users to insurance/loans</t>
+        </is>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr"/>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K87" s="5" t="inlineStr"/>
+      <c r="L87" s="5" t="inlineStr">
+        <is>
+          <t>$9M+; regulated marketplace</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Anyfin</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr"/>
+      <c r="D88" s="5" t="inlineStr"/>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Stockholm SE</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Fintech</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>AI consumer loan refinancing/assessment</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>agent-research</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr"/>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="K88" s="5" t="inlineStr"/>
+      <c r="L88" s="5" t="inlineStr">
+        <is>
+          <t>Multi-market; ~205 staff</t>
         </is>
       </c>
     </row>

</xml_diff>